<commit_message>
Add suplementary with others DLM
</commit_message>
<xml_diff>
--- a/Output/Correlation_exposure_table.xlsx
+++ b/Output/Correlation_exposure_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uccl0-my.sharepoint.com/personal/estela_blanco_uc_cl/Documents/Contaminación_Malformaciones Congénitas/Pollution_Malformation_TEM/Output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_54184E34035CA082CE475652F37BD2728A496552" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{597A1546-3B45-8840-9658-5F0137CE35FD}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_54184E34035CA082CE475652F37BD2728A496552" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00F3A572-C90E-BC45-B1C8-669AE0787F6A}"/>
   <bookViews>
-    <workbookView xWindow="-1640" yWindow="-21600" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1340" windowWidth="34560" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary_statistics_correlations" sheetId="1" r:id="rId1"/>
@@ -676,31 +676,31 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <v>5.0999999999999996</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>324.2</v>
+        <v>1.2</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0.19</v>
+        <v>0.06</v>
       </c>
       <c r="H6">
-        <v>-0.69</v>
+        <v>-0.89</v>
       </c>
       <c r="I6">
-        <v>0.11</v>
+        <v>-0.01</v>
       </c>
       <c r="J6" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="K6" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -711,31 +711,31 @@
         <v>0</v>
       </c>
       <c r="C7">
-        <v>5.4</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>281.8</v>
+        <v>1.2</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F7">
-        <v>0.19</v>
+        <v>0.06</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
       <c r="H7">
-        <v>0.08</v>
+        <v>-0.08</v>
       </c>
       <c r="I7">
-        <v>-0.69</v>
+        <v>-0.88</v>
       </c>
       <c r="J7" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="K7" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
@@ -746,31 +746,31 @@
         <v>0</v>
       </c>
       <c r="C8">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="D8">
-        <v>315</v>
+        <v>1.2</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F8">
-        <v>-0.69</v>
+        <v>-0.89</v>
       </c>
       <c r="G8">
-        <v>0.08</v>
+        <v>-0.08</v>
       </c>
       <c r="H8">
         <v>1</v>
       </c>
       <c r="I8">
-        <v>0.14000000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="J8" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="K8" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
@@ -781,31 +781,31 @@
         <v>70</v>
       </c>
       <c r="C9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>296.2</v>
+        <v>1.8</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="F9">
-        <v>0.11</v>
+        <v>-0.01</v>
       </c>
       <c r="G9">
-        <v>-0.69</v>
+        <v>-0.88</v>
       </c>
       <c r="H9">
-        <v>0.14000000000000001</v>
+        <v>0.02</v>
       </c>
       <c r="I9">
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="K9" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
@@ -816,28 +816,28 @@
         <v>6</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D10">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
       <c r="G10">
-        <v>0.06</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H10">
         <v>-0.89</v>
       </c>
       <c r="I10">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K10" t="s">
         <v>14</v>
@@ -851,28 +851,28 @@
         <v>0</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D11">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E11" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F11">
-        <v>0.06</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
       <c r="H11">
-        <v>-0.08</v>
+        <v>-0.06</v>
       </c>
       <c r="I11">
         <v>-0.88</v>
       </c>
       <c r="J11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K11" t="s">
         <v>14</v>
@@ -886,28 +886,28 @@
         <v>0</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D12">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="E12" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F12">
         <v>-0.89</v>
       </c>
       <c r="G12">
-        <v>-0.08</v>
+        <v>-0.06</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
       <c r="I12">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="J12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K12" t="s">
         <v>14</v>
@@ -921,28 +921,28 @@
         <v>70</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D13">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
       <c r="E13" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F13">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="G13">
         <v>-0.88</v>
       </c>
       <c r="H13">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="I13">
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K13" t="s">
         <v>14</v>
@@ -956,28 +956,28 @@
         <v>6</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="D14">
-        <v>1.6</v>
+        <v>324.2</v>
       </c>
       <c r="E14" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
       <c r="G14">
-        <v>0.08</v>
+        <v>0.19</v>
       </c>
       <c r="H14">
-        <v>-0.85</v>
+        <v>-0.69</v>
       </c>
       <c r="I14">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
       <c r="J14" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="K14" t="s">
         <v>28</v>
@@ -991,28 +991,28 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="D15">
-        <v>1.6</v>
+        <v>281.8</v>
       </c>
       <c r="E15" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F15">
+        <v>0.19</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
         <v>0.08</v>
       </c>
-      <c r="G15">
-        <v>1</v>
-      </c>
-      <c r="H15">
-        <v>-0.04</v>
-      </c>
       <c r="I15">
-        <v>-0.84</v>
+        <v>-0.69</v>
       </c>
       <c r="J15" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="K15" t="s">
         <v>28</v>
@@ -1026,28 +1026,28 @@
         <v>0</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="D16">
-        <v>1.6</v>
+        <v>315</v>
       </c>
       <c r="E16" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F16">
-        <v>-0.85</v>
+        <v>-0.69</v>
       </c>
       <c r="G16">
-        <v>-0.04</v>
+        <v>0.08</v>
       </c>
       <c r="H16">
         <v>1</v>
       </c>
       <c r="I16">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="J16" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="K16" t="s">
         <v>28</v>
@@ -1061,28 +1061,28 @@
         <v>70</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D17">
-        <v>2</v>
+        <v>296.2</v>
       </c>
       <c r="E17" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F17">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
       <c r="G17">
-        <v>-0.84</v>
+        <v>-0.69</v>
       </c>
       <c r="H17">
-        <v>0.05</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="I17">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="K17" t="s">
         <v>28</v>
@@ -1096,31 +1096,31 @@
         <v>6</v>
       </c>
       <c r="C18">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D18">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F18">
         <v>1</v>
       </c>
       <c r="G18">
-        <v>7.0000000000000007E-2</v>
+        <v>0.08</v>
       </c>
       <c r="H18">
-        <v>-0.89</v>
+        <v>-0.85</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="J18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K18" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
@@ -1131,31 +1131,31 @@
         <v>0</v>
       </c>
       <c r="C19">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D19">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E19" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F19">
-        <v>7.0000000000000007E-2</v>
+        <v>0.08</v>
       </c>
       <c r="G19">
         <v>1</v>
       </c>
       <c r="H19">
-        <v>-0.06</v>
+        <v>-0.04</v>
       </c>
       <c r="I19">
-        <v>-0.88</v>
+        <v>-0.84</v>
       </c>
       <c r="J19" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K19" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
@@ -1166,31 +1166,31 @@
         <v>0</v>
       </c>
       <c r="C20">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D20">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="E20" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="F20">
-        <v>-0.89</v>
+        <v>-0.85</v>
       </c>
       <c r="G20">
-        <v>-0.06</v>
+        <v>-0.04</v>
       </c>
       <c r="H20">
         <v>1</v>
       </c>
       <c r="I20">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="J20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K20" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
@@ -1201,31 +1201,31 @@
         <v>70</v>
       </c>
       <c r="C21">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="E21" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="G21">
-        <v>-0.88</v>
+        <v>-0.84</v>
       </c>
       <c r="H21">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="I21">
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K21" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
@@ -1371,7 +1371,7 @@
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K25">
-      <sortCondition descending="1" ref="J1:J25"/>
+      <sortCondition descending="1" ref="K1:K25"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>